<commit_message>
update sex column - remove mixed and add both - update data dictionary
</commit_message>
<xml_diff>
--- a/www/data-entry-template/GLATAR_data_entry_template_v19.xlsx
+++ b/www/data-entry-template/GLATAR_data_entry_template_v19.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/benhlina/Library/CloudStorage/Dropbox/GitHub/GLATAR-App/www/data-entry-template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0863B693-A905-4849-9C7A-9504CB1D5198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28408B8D-0B69-8A48-AC5B-3B9CE8B4732D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="640" windowWidth="34560" windowHeight="19460" xr2:uid="{DE6F8925-643B-304C-8933-23D4A9123DA3}"/>
   </bookViews>
@@ -44062,9 +44062,6 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="R6:R999" xr:uid="{C1262AB6-4400-D04A-976B-8F918C2989AD}">
       <formula1>"Total, Fork, Standard, Carapace"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L6:L999" xr:uid="{8B693881-68ED-E14E-BF9E-57D22ABE1721}">
-      <formula1>"male, female, unknown, mixed"</formula1>
-    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6:F999" xr:uid="{DF355696-A0A3-6D45-A97F-2A26E0345658}">
       <formula1>"spring, summer, fall, winter"</formula1>
     </dataValidation>
@@ -44095,6 +44092,9 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M6:M10000" xr:uid="{D77F31B9-1615-2E41-A61E-3373EC534A30}">
       <formula1>"fry, larva, nymph, pupa, juvenile, adult "</formula1>
     </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L6:L10000" xr:uid="{8E9C54B4-F117-8C42-9731-37E4B818ABAE}">
+      <formula1>"male, female, unknown, both"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>

</xml_diff>

<commit_message>
minor update to data_dictionary
</commit_message>
<xml_diff>
--- a/www/data-entry-template/GLATAR_data_entry_template_v19.xlsx
+++ b/www/data-entry-template/GLATAR_data_entry_template_v19.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/benhlina/Library/CloudStorage/Dropbox/GitHub/GLATAR-App/www/data-entry-template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28408B8D-0B69-8A48-AC5B-3B9CE8B4732D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D4FCCDD-1209-4C4D-A32A-CB76A590C72F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="640" windowWidth="34560" windowHeight="19460" xr2:uid="{DE6F8925-643B-304C-8933-23D4A9123DA3}"/>
   </bookViews>
@@ -526,9 +526,6 @@
     <t>doi</t>
   </si>
   <si>
-    <t>tbl_source</t>
-  </si>
-  <si>
     <t>as in: Timothy B. Johnson; format: character</t>
   </si>
   <si>
@@ -763,9 +760,6 @@
     <t>Journal volume number</t>
   </si>
   <si>
-    <t>tbl_source;tbl_samples</t>
-  </si>
-  <si>
     <t>as in: Journal Article; format: character</t>
   </si>
   <si>
@@ -943,9 +937,6 @@
     <t>as in: Benjamin L. Hlina; format: character</t>
   </si>
   <si>
-    <t>This data dictionary is to guide you in filling out/interpreting the fields in tbl_submission, tbl_source,  and tbl_samples data sheet. This sheet does not need to be submitted with your data. Green fields are required when submitting the data</t>
-  </si>
-  <si>
     <t>as in: juvenile - (i.e., fry, larva, juvenile, and adult); format: character</t>
   </si>
   <si>
@@ -1052,6 +1043,15 @@
   </si>
   <si>
     <t>Whether the sample is an Individual, Composite, Mean, SD, or Equation</t>
+  </si>
+  <si>
+    <t>tbl_sources</t>
+  </si>
+  <si>
+    <t>tbl_sources;tbl_samples</t>
+  </si>
+  <si>
+    <t>This data dictionary is to guide you in filling out/interpreting the fields in tbl_submission, tbl_sources,  and tbl_samples data sheet. This sheet does not need to be submitted with your data. Green fields are required when submitting the data</t>
   </si>
 </sst>
 </file>
@@ -1740,7 +1740,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="43" t="s">
-        <v>216</v>
+        <v>238</v>
       </c>
       <c r="B1" s="43"/>
       <c r="C1" s="43"/>
@@ -1748,7 +1748,7 @@
     </row>
     <row r="2" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="43" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B2" s="43"/>
       <c r="C2" s="43"/>
@@ -1770,49 +1770,49 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="23" t="s">
+        <v>209</v>
+      </c>
+      <c r="B5" s="24" t="s">
+        <v>205</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>213</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" s="23" t="s">
+        <v>209</v>
+      </c>
+      <c r="B6" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>189</v>
+      </c>
+      <c r="D6" s="25" t="s">
         <v>211</v>
       </c>
-      <c r="B5" s="24" t="s">
+    </row>
+    <row r="7" spans="1:4" ht="56" x14ac:dyDescent="0.2">
+      <c r="A7" s="23" t="s">
+        <v>209</v>
+      </c>
+      <c r="B7" s="24" t="s">
         <v>207</v>
       </c>
-      <c r="C5" s="9" t="s">
-        <v>215</v>
+      <c r="C7" s="19" t="s">
+        <v>171</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D7" s="25" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="23" t="s">
-        <v>211</v>
-      </c>
-      <c r="B6" s="24" t="s">
-        <v>208</v>
-      </c>
-      <c r="C6" s="19" t="s">
-        <v>191</v>
-      </c>
-      <c r="D6" s="25" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="56" x14ac:dyDescent="0.2">
-      <c r="A7" s="23" t="s">
-        <v>211</v>
-      </c>
-      <c r="B7" s="24" t="s">
-        <v>209</v>
-      </c>
-      <c r="C7" s="19" t="s">
-        <v>173</v>
-      </c>
-      <c r="D7" s="25" t="s">
-        <v>214</v>
-      </c>
-    </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" s="26" t="s">
-        <v>156</v>
+        <v>237</v>
       </c>
       <c r="B8" s="27" t="s">
         <v>4</v>
@@ -1821,214 +1821,214 @@
         <v>66</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="28" x14ac:dyDescent="0.2">
       <c r="A9" s="26" t="s">
-        <v>89</v>
+        <v>236</v>
       </c>
       <c r="B9" s="28" t="s">
         <v>79</v>
       </c>
       <c r="C9" s="25" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="28" x14ac:dyDescent="0.2">
       <c r="A10" s="26" t="s">
-        <v>89</v>
+        <v>236</v>
       </c>
       <c r="B10" s="28" t="s">
         <v>80</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="D10" s="25" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="56" x14ac:dyDescent="0.2">
       <c r="A11" s="26" t="s">
-        <v>89</v>
+        <v>236</v>
       </c>
       <c r="B11" s="25" t="s">
         <v>81</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D11" s="25" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" s="26" t="s">
-        <v>89</v>
+        <v>236</v>
       </c>
       <c r="B12" s="28" t="s">
         <v>82</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D12" s="25" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="28" x14ac:dyDescent="0.2">
       <c r="A13" s="26" t="s">
-        <v>89</v>
+        <v>236</v>
       </c>
       <c r="B13" s="25" t="s">
         <v>83</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D13" s="25" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14" s="26" t="s">
+        <v>236</v>
+      </c>
+      <c r="B14" s="28" t="s">
+        <v>132</v>
+      </c>
+      <c r="C14" s="25" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="26" t="s">
-        <v>89</v>
-      </c>
-      <c r="B14" s="28" t="s">
-        <v>133</v>
-      </c>
-      <c r="C14" s="25" t="s">
+      <c r="D14" s="25" t="s">
         <v>97</v>
       </c>
-      <c r="D14" s="25" t="s">
-        <v>98</v>
-      </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" s="26" t="s">
-        <v>89</v>
+        <v>236</v>
       </c>
       <c r="B15" s="25" t="s">
         <v>84</v>
       </c>
       <c r="C15" s="25" t="s">
+        <v>175</v>
+      </c>
+      <c r="D15" s="25" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" s="26" t="s">
+        <v>236</v>
+      </c>
+      <c r="B16" s="25" t="s">
+        <v>133</v>
+      </c>
+      <c r="C16" s="25" t="s">
+        <v>152</v>
+      </c>
+      <c r="D16" s="25" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17" s="26" t="s">
+        <v>236</v>
+      </c>
+      <c r="B17" s="25" t="s">
+        <v>134</v>
+      </c>
+      <c r="C17" s="25" t="s">
         <v>177</v>
       </c>
-      <c r="D15" s="25" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="26" t="s">
-        <v>89</v>
-      </c>
-      <c r="B16" s="25" t="s">
-        <v>134</v>
-      </c>
-      <c r="C16" s="25" t="s">
+      <c r="D17" s="25" t="s">
         <v>153</v>
       </c>
-      <c r="D16" s="25" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="26" t="s">
-        <v>89</v>
-      </c>
-      <c r="B17" s="25" t="s">
-        <v>135</v>
-      </c>
-      <c r="C17" s="25" t="s">
-        <v>179</v>
-      </c>
-      <c r="D17" s="25" t="s">
-        <v>154</v>
-      </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" s="26" t="s">
-        <v>89</v>
+        <v>236</v>
       </c>
       <c r="B18" s="25" t="s">
         <v>85</v>
       </c>
       <c r="C18" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="D18" s="25" t="s">
         <v>100</v>
       </c>
-      <c r="D18" s="25" t="s">
-        <v>101</v>
-      </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" s="26" t="s">
-        <v>89</v>
+        <v>236</v>
       </c>
       <c r="B19" s="25" t="s">
         <v>86</v>
       </c>
       <c r="C19" s="25" t="s">
+        <v>101</v>
+      </c>
+      <c r="D19" s="25" t="s">
         <v>102</v>
       </c>
-      <c r="D19" s="25" t="s">
-        <v>103</v>
-      </c>
     </row>
     <row r="20" spans="1:4" ht="28" x14ac:dyDescent="0.2">
       <c r="A20" s="26" t="s">
-        <v>89</v>
+        <v>236</v>
       </c>
       <c r="B20" s="25" t="s">
         <v>87</v>
       </c>
       <c r="C20" s="19" t="s">
+        <v>103</v>
+      </c>
+      <c r="D20" s="25" t="s">
         <v>104</v>
       </c>
-      <c r="D20" s="25" t="s">
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A21" s="26" t="s">
+        <v>236</v>
+      </c>
+      <c r="B21" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="C21" s="19" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" s="26" t="s">
-        <v>89</v>
-      </c>
-      <c r="B21" s="25" t="s">
-        <v>167</v>
-      </c>
-      <c r="C21" s="19" t="s">
+      <c r="D21" s="25" t="s">
         <v>106</v>
       </c>
-      <c r="D21" s="25" t="s">
-        <v>107</v>
-      </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" s="26" t="s">
-        <v>89</v>
+        <v>236</v>
       </c>
       <c r="B22" s="25" t="s">
         <v>88</v>
       </c>
       <c r="C22" s="25" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D22" s="25" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" s="29" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B23" s="30" t="s">
         <v>14</v>
       </c>
       <c r="C23" s="20" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D23" s="20" t="s">
         <v>18</v>
@@ -2036,10 +2036,10 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" s="31" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B24" s="31" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C24" s="31" t="s">
         <v>40</v>
@@ -2050,69 +2050,69 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" s="31" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B25" s="32" t="s">
         <v>70</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" s="31" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B26" s="31" t="s">
         <v>5</v>
       </c>
       <c r="C26" s="31" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="D26" s="31" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" s="31" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B27" s="31" t="s">
+        <v>110</v>
+      </c>
+      <c r="C27" s="31" t="s">
+        <v>183</v>
+      </c>
+      <c r="D27" s="31" t="s">
         <v>111</v>
       </c>
-      <c r="C27" s="31" t="s">
-        <v>185</v>
-      </c>
-      <c r="D27" s="31" t="s">
-        <v>112</v>
-      </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" s="31" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B28" s="31" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C28" s="31" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D28" s="31" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" s="31" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B29" s="33" t="s">
         <v>6</v>
       </c>
       <c r="C29" s="31" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D29" s="31" t="s">
         <v>11</v>
@@ -2120,55 +2120,55 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" s="31" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B30" s="33" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C30" s="31" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D30" s="31" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" s="31" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B31" s="31" t="s">
         <v>15</v>
       </c>
       <c r="C31" s="31" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="D31" s="31" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A32" s="31" t="s">
+        <v>141</v>
+      </c>
+      <c r="B32" s="31" t="s">
+        <v>123</v>
+      </c>
+      <c r="C32" s="31" t="s">
+        <v>162</v>
+      </c>
+      <c r="D32" s="31" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A32" s="31" t="s">
-        <v>142</v>
-      </c>
-      <c r="B32" s="31" t="s">
-        <v>124</v>
-      </c>
-      <c r="C32" s="31" t="s">
-        <v>164</v>
-      </c>
-      <c r="D32" s="31" t="s">
-        <v>128</v>
-      </c>
-    </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" s="31" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B33" s="31" t="s">
         <v>7</v>
       </c>
       <c r="C33" s="31" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="D33" s="31" t="s">
         <v>41</v>
@@ -2176,21 +2176,21 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" s="31" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B34" s="31" t="s">
         <v>8</v>
       </c>
       <c r="C34" s="31" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="D34" s="31" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" s="31" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B35" s="33" t="s">
         <v>13</v>
@@ -2199,29 +2199,29 @@
         <v>50</v>
       </c>
       <c r="D35" s="34" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="28" x14ac:dyDescent="0.2">
       <c r="A36" s="31" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B36" s="31" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C36" s="31" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="D36" s="34" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" s="31" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B37" s="31" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C37" s="31" t="s">
         <v>49</v>
@@ -2232,66 +2232,66 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" s="31" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B38" s="31" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C38" s="31" t="s">
         <v>51</v>
       </c>
       <c r="D38" s="31" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="28" x14ac:dyDescent="0.2">
       <c r="A39" s="31" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B39" s="31" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C39" s="31" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D39" s="34" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40" s="31" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B40" s="31" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C40" s="31" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D40" s="31" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="28" x14ac:dyDescent="0.2">
       <c r="A41" s="31" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B41" s="33" t="s">
+        <v>232</v>
+      </c>
+      <c r="C41" s="31" t="s">
+        <v>234</v>
+      </c>
+      <c r="D41" s="34" t="s">
         <v>235</v>
       </c>
-      <c r="C41" s="31" t="s">
-        <v>237</v>
-      </c>
-      <c r="D41" s="34" t="s">
-        <v>238</v>
-      </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" s="31" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B42" s="31" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="C42" s="31" t="s">
         <v>72</v>
@@ -2302,7 +2302,7 @@
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43" s="31" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B43" s="33" t="s">
         <v>9</v>
@@ -2316,7 +2316,7 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44" s="31" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B44" s="33" t="s">
         <v>75</v>
@@ -2333,13 +2333,13 @@
         <v>16</v>
       </c>
       <c r="B45" s="31" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C45" s="31" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D45" s="31" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
@@ -2364,10 +2364,10 @@
         <v>19</v>
       </c>
       <c r="C47" s="31" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="D47" s="31" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
@@ -2381,7 +2381,7 @@
         <v>60</v>
       </c>
       <c r="D48" s="31" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
@@ -2392,7 +2392,7 @@
         <v>21</v>
       </c>
       <c r="C49" s="31" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="D49" s="31" t="s">
         <v>61</v>
@@ -2406,7 +2406,7 @@
         <v>22</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="D50" s="3" t="s">
         <v>26</v>
@@ -2420,10 +2420,10 @@
         <v>23</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
@@ -2445,13 +2445,13 @@
         <v>28</v>
       </c>
       <c r="B53" s="35" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
@@ -2459,13 +2459,13 @@
         <v>28</v>
       </c>
       <c r="B54" s="31" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C54" s="31" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D54" s="31" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
@@ -2473,13 +2473,13 @@
         <v>28</v>
       </c>
       <c r="B55" s="31" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C55" s="31" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="D55" s="31" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
@@ -2487,13 +2487,13 @@
         <v>28</v>
       </c>
       <c r="B56" s="31" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C56" s="31" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D56" s="31" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
@@ -2501,13 +2501,13 @@
         <v>28</v>
       </c>
       <c r="B57" s="21" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C57" s="31" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="D57" s="31" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
@@ -2515,13 +2515,13 @@
         <v>28</v>
       </c>
       <c r="B58" s="31" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C58" s="31" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D58" s="31" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.2">
@@ -2529,13 +2529,13 @@
         <v>28</v>
       </c>
       <c r="B59" s="31" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C59" s="31" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D59" s="31" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="60" spans="1:4" ht="28" x14ac:dyDescent="0.2">
@@ -2543,13 +2543,13 @@
         <v>28</v>
       </c>
       <c r="B60" s="21" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C60" s="31" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D60" s="34" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="28" x14ac:dyDescent="0.2">
@@ -2557,13 +2557,13 @@
         <v>28</v>
       </c>
       <c r="B61" s="21" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C61" s="31" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D61" s="34" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
@@ -2655,13 +2655,13 @@
         <v>39</v>
       </c>
       <c r="B68" s="21" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="C68" s="31" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="D68" s="34" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.2">
@@ -2711,13 +2711,13 @@
         <v>39</v>
       </c>
       <c r="B72" s="31" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="C72" s="31" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="D72" s="31" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.2">
@@ -2725,13 +2725,13 @@
         <v>39</v>
       </c>
       <c r="B73" s="31" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C73" s="31" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="D73" s="31" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.2">
@@ -2739,13 +2739,13 @@
         <v>39</v>
       </c>
       <c r="B74" s="31" t="s">
+        <v>149</v>
+      </c>
+      <c r="C74" s="31" t="s">
         <v>150</v>
       </c>
-      <c r="C74" s="31" t="s">
+      <c r="D74" s="31" t="s">
         <v>151</v>
-      </c>
-      <c r="D74" s="31" t="s">
-        <v>152</v>
       </c>
     </row>
   </sheetData>
@@ -2769,12 +2769,12 @@
   <sheetData>
     <row r="1" spans="1:4" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="44" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="B1" s="45"/>
       <c r="C1" s="45"/>
       <c r="D1" s="10" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
@@ -2790,18 +2790,18 @@
       <c r="B3" s="44"/>
       <c r="C3" s="44"/>
       <c r="D3" s="11" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="13" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
@@ -2835,12 +2835,12 @@
   <sheetData>
     <row r="1" spans="1:15" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="44" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B1" s="45"/>
       <c r="C1" s="45"/>
       <c r="D1" s="10" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.2">
@@ -2861,7 +2861,7 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" s="15" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B4" s="16" t="s">
         <v>79</v>
@@ -2879,16 +2879,16 @@
         <v>83</v>
       </c>
       <c r="G4" s="16" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>84</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>85</v>
@@ -2900,7 +2900,7 @@
         <v>87</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="O4" s="2" t="s">
         <v>88</v>
@@ -43847,12 +43847,12 @@
   <sheetData>
     <row r="1" spans="1:53" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="44" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B1" s="45"/>
       <c r="C1" s="45"/>
       <c r="D1" s="5" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
     </row>
     <row r="2" spans="1:53" x14ac:dyDescent="0.2">
@@ -43873,7 +43873,7 @@
     </row>
     <row r="4" spans="1:53" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="X4" t="s">
         <v>16</v>
@@ -43896,34 +43896,34 @@
         <v>78</v>
       </c>
       <c r="C5" s="37" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D5" s="38" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="E5" s="37" t="s">
         <v>65</v>
       </c>
       <c r="F5" s="37" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G5" s="37" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H5" s="39" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="I5" s="39" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="J5" s="37" t="s">
         <v>15</v>
       </c>
       <c r="K5" s="37" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="L5" s="37" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="M5" s="37" t="s">
         <v>8</v>
@@ -43932,25 +43932,25 @@
         <v>13</v>
       </c>
       <c r="O5" s="37" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="P5" s="37" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="Q5" s="37" t="s">
+        <v>112</v>
+      </c>
+      <c r="R5" s="37" t="s">
         <v>113</v>
       </c>
-      <c r="R5" s="37" t="s">
-        <v>114</v>
-      </c>
       <c r="S5" s="37" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="T5" s="40" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="U5" s="40" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="V5" s="39" t="s">
         <v>9</v>
@@ -43959,7 +43959,7 @@
         <v>71</v>
       </c>
       <c r="X5" s="40" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="Y5" s="39" t="s">
         <v>17</v>
@@ -43974,40 +43974,40 @@
         <v>21</v>
       </c>
       <c r="AC5" s="42" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="AD5" s="42" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="AE5" s="42" t="s">
         <v>67</v>
       </c>
       <c r="AF5" s="42" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="AG5" s="37" t="s">
+        <v>138</v>
+      </c>
+      <c r="AH5" s="37" t="s">
+        <v>114</v>
+      </c>
+      <c r="AI5" s="37" t="s">
+        <v>142</v>
+      </c>
+      <c r="AJ5" s="37" t="s">
+        <v>115</v>
+      </c>
+      <c r="AK5" s="40" t="s">
         <v>139</v>
       </c>
-      <c r="AH5" s="37" t="s">
-        <v>115</v>
+      <c r="AL5" s="40" t="s">
+        <v>140</v>
       </c>
-      <c r="AI5" s="37" t="s">
+      <c r="AM5" s="40" t="s">
         <v>143</v>
       </c>
-      <c r="AJ5" s="37" t="s">
-        <v>116</v>
-      </c>
-      <c r="AK5" s="40" t="s">
-        <v>140</v>
-      </c>
-      <c r="AL5" s="40" t="s">
-        <v>141</v>
-      </c>
-      <c r="AM5" s="40" t="s">
+      <c r="AN5" s="40" t="s">
         <v>144</v>
-      </c>
-      <c r="AN5" s="40" t="s">
-        <v>145</v>
       </c>
       <c r="AO5" s="37" t="s">
         <v>29</v>
@@ -44028,7 +44028,7 @@
         <v>35</v>
       </c>
       <c r="AU5" s="37" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="AV5" s="37" t="s">
         <v>36</v>
@@ -44040,13 +44040,13 @@
         <v>38</v>
       </c>
       <c r="AY5" s="37" t="s">
+        <v>226</v>
+      </c>
+      <c r="AZ5" s="37" t="s">
         <v>229</v>
       </c>
-      <c r="AZ5" s="37" t="s">
-        <v>232</v>
-      </c>
       <c r="BA5" s="37" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
   </sheetData>

</xml_diff>